<commit_message>
vault backup: 2026-05-31 12:07:01
</commit_message>
<xml_diff>
--- a/linkedin-inbound-outlook.xlsx
+++ b/linkedin-inbound-outlook.xlsx
@@ -365,56 +365,60 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -422,35 +426,35 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -721,700 +725,700 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="15"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="B4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>556</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="B7" s="7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <f aca="false">52/12</f>
         <v>4.33333333333333</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>0.75</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="8" t="n">
         <v>0.55</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="11" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <v>0.001</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="11" t="n">
         <v>0.002</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <v>0.003</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="8" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="8" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="13" t="n">
         <f aca="false">B7*B9*B8+B11</f>
-        <v>60.1666666666667</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+        <v>114.333333333333</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="13" t="n">
         <f aca="false">B7*B9*B8*B10+B11*B12</f>
-        <v>43.625</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+        <v>84.25</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F26" s="13" t="s">
+      <c r="F26" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G26" s="13" t="s">
+      <c r="G26" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="14" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="B27" s="15" t="n">
+      <c r="B27" s="16" t="n">
         <f aca="false">B5</f>
         <v>556</v>
       </c>
-      <c r="C27" s="15" t="n">
+      <c r="C27" s="16" t="n">
         <f aca="false">B5*B6</f>
         <v>139</v>
       </c>
-      <c r="D27" s="16" t="n">
+      <c r="D27" s="17" t="n">
         <f aca="false">C27/B27</f>
         <v>0.25</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E27" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="H27" s="18" t="n">
+      <c r="H27" s="19" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B28" s="15" t="n">
+      <c r="B28" s="16" t="n">
         <f aca="false">B27+$B$22</f>
-        <v>616.166666666667</v>
-      </c>
-      <c r="C28" s="15" t="n">
+        <v>670.333333333333</v>
+      </c>
+      <c r="C28" s="16" t="n">
         <f aca="false">C27+$B$23</f>
-        <v>182.625</v>
-      </c>
-      <c r="D28" s="16" t="n">
+        <v>223.25</v>
+      </c>
+      <c r="D28" s="17" t="n">
         <f aca="false">C28/B28</f>
-        <v>0.296388964024885</v>
-      </c>
-      <c r="E28" s="15" t="n">
+        <v>0.333043262058677</v>
+      </c>
+      <c r="E28" s="16" t="n">
         <f aca="false">C28*$B$13</f>
-        <v>100.44375</v>
-      </c>
-      <c r="F28" s="17" t="n">
+        <v>122.7875</v>
+      </c>
+      <c r="F28" s="18" t="n">
         <f aca="false">IF(A28&lt;=3,$B$14,IF(A28&lt;=6,$B$15,IF(A28&lt;=9,$B$16,$B$17)))</f>
         <v>0</v>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G28" s="9" t="n">
         <f aca="false">E28*F28</f>
         <v>0</v>
       </c>
-      <c r="H28" s="18" t="n">
+      <c r="H28" s="19" t="n">
         <f aca="false">H27+G28</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B29" s="15" t="n">
+      <c r="B29" s="16" t="n">
         <f aca="false">B28+$B$22</f>
-        <v>676.333333333333</v>
-      </c>
-      <c r="C29" s="15" t="n">
+        <v>784.666666666667</v>
+      </c>
+      <c r="C29" s="16" t="n">
         <f aca="false">C28+$B$23</f>
-        <v>226.25</v>
-      </c>
-      <c r="D29" s="16" t="n">
+        <v>307.5</v>
+      </c>
+      <c r="D29" s="17" t="n">
         <f aca="false">C29/B29</f>
-        <v>0.334524396254313</v>
-      </c>
-      <c r="E29" s="15" t="n">
+        <v>0.391886151231946</v>
+      </c>
+      <c r="E29" s="16" t="n">
         <f aca="false">C29*$B$13</f>
-        <v>124.4375</v>
-      </c>
-      <c r="F29" s="17" t="n">
+        <v>169.125</v>
+      </c>
+      <c r="F29" s="18" t="n">
         <f aca="false">IF(A29&lt;=3,$B$14,IF(A29&lt;=6,$B$15,IF(A29&lt;=9,$B$16,$B$17)))</f>
         <v>0</v>
       </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="9" t="n">
         <f aca="false">E29*F29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="18" t="n">
+      <c r="H29" s="19" t="n">
         <f aca="false">H28+G29</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B30" s="16" t="n">
         <f aca="false">B29+$B$22</f>
-        <v>736.5</v>
-      </c>
-      <c r="C30" s="15" t="n">
+        <v>899</v>
+      </c>
+      <c r="C30" s="16" t="n">
         <f aca="false">C29+$B$23</f>
-        <v>269.875</v>
-      </c>
-      <c r="D30" s="16" t="n">
+        <v>391.75</v>
+      </c>
+      <c r="D30" s="17" t="n">
         <f aca="false">C30/B30</f>
-        <v>0.36642905634759</v>
-      </c>
-      <c r="E30" s="15" t="n">
+        <v>0.435761957730812</v>
+      </c>
+      <c r="E30" s="16" t="n">
         <f aca="false">C30*$B$13</f>
-        <v>148.43125</v>
-      </c>
-      <c r="F30" s="17" t="n">
+        <v>215.4625</v>
+      </c>
+      <c r="F30" s="18" t="n">
         <f aca="false">IF(A30&lt;=3,$B$14,IF(A30&lt;=6,$B$15,IF(A30&lt;=9,$B$16,$B$17)))</f>
         <v>0</v>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="9" t="n">
         <f aca="false">E30*F30</f>
         <v>0</v>
       </c>
-      <c r="H30" s="18" t="n">
+      <c r="H30" s="19" t="n">
         <f aca="false">H29+G30</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B31" s="15" t="n">
+      <c r="B31" s="16" t="n">
         <f aca="false">B30+$B$22</f>
-        <v>796.666666666667</v>
-      </c>
-      <c r="C31" s="15" t="n">
+        <v>1013.33333333333</v>
+      </c>
+      <c r="C31" s="16" t="n">
         <f aca="false">C30+$B$23</f>
-        <v>313.5</v>
-      </c>
-      <c r="D31" s="16" t="n">
+        <v>476</v>
+      </c>
+      <c r="D31" s="17" t="n">
         <f aca="false">C31/B31</f>
-        <v>0.393514644351465</v>
-      </c>
-      <c r="E31" s="15" t="n">
+        <v>0.469736842105263</v>
+      </c>
+      <c r="E31" s="16" t="n">
         <f aca="false">C31*$B$13</f>
-        <v>172.425</v>
-      </c>
-      <c r="F31" s="17" t="n">
+        <v>261.8</v>
+      </c>
+      <c r="F31" s="18" t="n">
         <f aca="false">IF(A31&lt;=3,$B$14,IF(A31&lt;=6,$B$15,IF(A31&lt;=9,$B$16,$B$17)))</f>
         <v>0.001</v>
       </c>
-      <c r="G31" s="8" t="n">
+      <c r="G31" s="9" t="n">
         <f aca="false">E31*F31</f>
-        <v>0.172425</v>
-      </c>
-      <c r="H31" s="18" t="n">
+        <v>0.2618</v>
+      </c>
+      <c r="H31" s="19" t="n">
         <f aca="false">H30+G31</f>
-        <v>0.172425</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="n">
+        <v>0.2618</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="16" t="n">
         <f aca="false">B31+$B$22</f>
-        <v>856.833333333333</v>
-      </c>
-      <c r="C32" s="15" t="n">
+        <v>1127.66666666667</v>
+      </c>
+      <c r="C32" s="16" t="n">
         <f aca="false">C31+$B$23</f>
-        <v>357.125</v>
-      </c>
-      <c r="D32" s="16" t="n">
+        <v>560.25</v>
+      </c>
+      <c r="D32" s="17" t="n">
         <f aca="false">C32/B32</f>
-        <v>0.416796343123906</v>
-      </c>
-      <c r="E32" s="15" t="n">
+        <v>0.496822347029264</v>
+      </c>
+      <c r="E32" s="16" t="n">
         <f aca="false">C32*$B$13</f>
-        <v>196.41875</v>
-      </c>
-      <c r="F32" s="17" t="n">
+        <v>308.1375</v>
+      </c>
+      <c r="F32" s="18" t="n">
         <f aca="false">IF(A32&lt;=3,$B$14,IF(A32&lt;=6,$B$15,IF(A32&lt;=9,$B$16,$B$17)))</f>
         <v>0.001</v>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="9" t="n">
         <f aca="false">E32*F32</f>
-        <v>0.19641875</v>
-      </c>
-      <c r="H32" s="18" t="n">
+        <v>0.3081375</v>
+      </c>
+      <c r="H32" s="19" t="n">
         <f aca="false">H31+G32</f>
-        <v>0.36884375</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="n">
+        <v>0.5699375</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B33" s="15" t="n">
+      <c r="B33" s="16" t="n">
         <f aca="false">B32+$B$22</f>
-        <v>917</v>
-      </c>
-      <c r="C33" s="15" t="n">
+        <v>1242</v>
+      </c>
+      <c r="C33" s="16" t="n">
         <f aca="false">C32+$B$23</f>
-        <v>400.75</v>
-      </c>
-      <c r="D33" s="16" t="n">
+        <v>644.5</v>
+      </c>
+      <c r="D33" s="17" t="n">
         <f aca="false">C33/B33</f>
-        <v>0.437022900763359</v>
-      </c>
-      <c r="E33" s="15" t="n">
+        <v>0.518921095008052</v>
+      </c>
+      <c r="E33" s="16" t="n">
         <f aca="false">C33*$B$13</f>
-        <v>220.4125</v>
-      </c>
-      <c r="F33" s="17" t="n">
+        <v>354.475</v>
+      </c>
+      <c r="F33" s="18" t="n">
         <f aca="false">IF(A33&lt;=3,$B$14,IF(A33&lt;=6,$B$15,IF(A33&lt;=9,$B$16,$B$17)))</f>
         <v>0.001</v>
       </c>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="9" t="n">
         <f aca="false">E33*F33</f>
-        <v>0.2204125</v>
-      </c>
-      <c r="H33" s="18" t="n">
+        <v>0.354475</v>
+      </c>
+      <c r="H33" s="19" t="n">
         <f aca="false">H32+G33</f>
-        <v>0.58925625</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14" t="n">
+        <v>0.9244125</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B34" s="15" t="n">
+      <c r="B34" s="16" t="n">
         <f aca="false">B33+$B$22</f>
-        <v>977.166666666666</v>
-      </c>
-      <c r="C34" s="15" t="n">
+        <v>1356.33333333333</v>
+      </c>
+      <c r="C34" s="16" t="n">
         <f aca="false">C33+$B$23</f>
-        <v>444.375</v>
-      </c>
-      <c r="D34" s="16" t="n">
+        <v>728.75</v>
+      </c>
+      <c r="D34" s="17" t="n">
         <f aca="false">C34/B34</f>
-        <v>0.454758655978168</v>
-      </c>
-      <c r="E34" s="15" t="n">
+        <v>0.537294175473089</v>
+      </c>
+      <c r="E34" s="16" t="n">
         <f aca="false">C34*$B$13</f>
-        <v>244.40625</v>
-      </c>
-      <c r="F34" s="17" t="n">
+        <v>400.8125</v>
+      </c>
+      <c r="F34" s="18" t="n">
         <f aca="false">IF(A34&lt;=3,$B$14,IF(A34&lt;=6,$B$15,IF(A34&lt;=9,$B$16,$B$17)))</f>
         <v>0.002</v>
       </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="9" t="n">
         <f aca="false">E34*F34</f>
-        <v>0.4888125</v>
-      </c>
-      <c r="H34" s="18" t="n">
+        <v>0.801625</v>
+      </c>
+      <c r="H34" s="19" t="n">
         <f aca="false">H33+G34</f>
-        <v>1.07806875</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="n">
+        <v>1.7260375</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B35" s="15" t="n">
+      <c r="B35" s="16" t="n">
         <f aca="false">B34+$B$22</f>
-        <v>1037.33333333333</v>
-      </c>
-      <c r="C35" s="15" t="n">
+        <v>1470.66666666667</v>
+      </c>
+      <c r="C35" s="16" t="n">
         <f aca="false">C34+$B$23</f>
-        <v>488</v>
-      </c>
-      <c r="D35" s="16" t="n">
+        <v>813</v>
+      </c>
+      <c r="D35" s="17" t="n">
         <f aca="false">C35/B35</f>
-        <v>0.470437017994859</v>
-      </c>
-      <c r="E35" s="15" t="n">
+        <v>0.552810516772439</v>
+      </c>
+      <c r="E35" s="16" t="n">
         <f aca="false">C35*$B$13</f>
-        <v>268.4</v>
-      </c>
-      <c r="F35" s="17" t="n">
+        <v>447.15</v>
+      </c>
+      <c r="F35" s="18" t="n">
         <f aca="false">IF(A35&lt;=3,$B$14,IF(A35&lt;=6,$B$15,IF(A35&lt;=9,$B$16,$B$17)))</f>
         <v>0.002</v>
       </c>
-      <c r="G35" s="8" t="n">
+      <c r="G35" s="9" t="n">
         <f aca="false">E35*F35</f>
-        <v>0.5368</v>
-      </c>
-      <c r="H35" s="18" t="n">
+        <v>0.8943</v>
+      </c>
+      <c r="H35" s="19" t="n">
         <f aca="false">H34+G35</f>
-        <v>1.61486875</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="n">
+        <v>2.6203375</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="B36" s="15" t="n">
+      <c r="B36" s="16" t="n">
         <f aca="false">B35+$B$22</f>
-        <v>1097.5</v>
-      </c>
-      <c r="C36" s="15" t="n">
+        <v>1585</v>
+      </c>
+      <c r="C36" s="16" t="n">
         <f aca="false">C35+$B$23</f>
-        <v>531.625</v>
-      </c>
-      <c r="D36" s="16" t="n">
+        <v>897.25</v>
+      </c>
+      <c r="D36" s="17" t="n">
         <f aca="false">C36/B36</f>
-        <v>0.484396355353075</v>
-      </c>
-      <c r="E36" s="15" t="n">
+        <v>0.56608832807571</v>
+      </c>
+      <c r="E36" s="16" t="n">
         <f aca="false">C36*$B$13</f>
-        <v>292.39375</v>
-      </c>
-      <c r="F36" s="17" t="n">
+        <v>493.4875</v>
+      </c>
+      <c r="F36" s="18" t="n">
         <f aca="false">IF(A36&lt;=3,$B$14,IF(A36&lt;=6,$B$15,IF(A36&lt;=9,$B$16,$B$17)))</f>
         <v>0.002</v>
       </c>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="9" t="n">
         <f aca="false">E36*F36</f>
-        <v>0.5847875</v>
-      </c>
-      <c r="H36" s="18" t="n">
+        <v>0.986975</v>
+      </c>
+      <c r="H36" s="19" t="n">
         <f aca="false">H35+G36</f>
-        <v>2.19965625</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="n">
+        <v>3.6073125</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B37" s="15" t="n">
+      <c r="B37" s="16" t="n">
         <f aca="false">B36+$B$22</f>
-        <v>1157.66666666667</v>
-      </c>
-      <c r="C37" s="15" t="n">
+        <v>1699.33333333333</v>
+      </c>
+      <c r="C37" s="16" t="n">
         <f aca="false">C36+$B$23</f>
-        <v>575.25</v>
-      </c>
-      <c r="D37" s="16" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="D37" s="17" t="n">
         <f aca="false">C37/B37</f>
-        <v>0.49690469334869</v>
-      </c>
-      <c r="E37" s="15" t="n">
+        <v>0.577579442918792</v>
+      </c>
+      <c r="E37" s="16" t="n">
         <f aca="false">C37*$B$13</f>
-        <v>316.3875</v>
-      </c>
-      <c r="F37" s="17" t="n">
+        <v>539.825</v>
+      </c>
+      <c r="F37" s="18" t="n">
         <f aca="false">IF(A37&lt;=3,$B$14,IF(A37&lt;=6,$B$15,IF(A37&lt;=9,$B$16,$B$17)))</f>
         <v>0.003</v>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="9" t="n">
         <f aca="false">E37*F37</f>
-        <v>0.9491625</v>
-      </c>
-      <c r="H37" s="18" t="n">
+        <v>1.619475</v>
+      </c>
+      <c r="H37" s="19" t="n">
         <f aca="false">H36+G37</f>
-        <v>3.14881875</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14" t="n">
+        <v>5.2267875</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="B38" s="15" t="n">
+      <c r="B38" s="16" t="n">
         <f aca="false">B37+$B$22</f>
-        <v>1217.83333333333</v>
-      </c>
-      <c r="C38" s="15" t="n">
+        <v>1813.66666666667</v>
+      </c>
+      <c r="C38" s="16" t="n">
         <f aca="false">C37+$B$23</f>
-        <v>618.875</v>
-      </c>
-      <c r="D38" s="16" t="n">
+        <v>1065.75</v>
+      </c>
+      <c r="D38" s="17" t="n">
         <f aca="false">C38/B38</f>
-        <v>0.508177090461202</v>
-      </c>
-      <c r="E38" s="15" t="n">
+        <v>0.587621760705753</v>
+      </c>
+      <c r="E38" s="16" t="n">
         <f aca="false">C38*$B$13</f>
-        <v>340.38125</v>
-      </c>
-      <c r="F38" s="17" t="n">
+        <v>586.1625</v>
+      </c>
+      <c r="F38" s="18" t="n">
         <f aca="false">IF(A38&lt;=3,$B$14,IF(A38&lt;=6,$B$15,IF(A38&lt;=9,$B$16,$B$17)))</f>
         <v>0.003</v>
       </c>
-      <c r="G38" s="8" t="n">
+      <c r="G38" s="9" t="n">
         <f aca="false">E38*F38</f>
-        <v>1.02114375</v>
-      </c>
-      <c r="H38" s="18" t="n">
+        <v>1.7584875</v>
+      </c>
+      <c r="H38" s="19" t="n">
         <f aca="false">H37+G38</f>
-        <v>4.1699625</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14" t="n">
+        <v>6.985275</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B39" s="15" t="n">
+      <c r="B39" s="16" t="n">
         <f aca="false">B38+$B$22</f>
-        <v>1278</v>
-      </c>
-      <c r="C39" s="15" t="n">
+        <v>1928</v>
+      </c>
+      <c r="C39" s="16" t="n">
         <f aca="false">C38+$B$23</f>
-        <v>662.5</v>
-      </c>
-      <c r="D39" s="16" t="n">
+        <v>1150</v>
+      </c>
+      <c r="D39" s="17" t="n">
         <f aca="false">C39/B39</f>
-        <v>0.518388106416275</v>
-      </c>
-      <c r="E39" s="15" t="n">
+        <v>0.596473029045643</v>
+      </c>
+      <c r="E39" s="16" t="n">
         <f aca="false">C39*$B$13</f>
-        <v>364.375</v>
-      </c>
-      <c r="F39" s="17" t="n">
+        <v>632.5</v>
+      </c>
+      <c r="F39" s="18" t="n">
         <f aca="false">IF(A39&lt;=3,$B$14,IF(A39&lt;=6,$B$15,IF(A39&lt;=9,$B$16,$B$17)))</f>
         <v>0.003</v>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="9" t="n">
         <f aca="false">E39*F39</f>
-        <v>1.093125</v>
-      </c>
-      <c r="H39" s="18" t="n">
+        <v>1.8975</v>
+      </c>
+      <c r="H39" s="19" t="n">
         <f aca="false">H38+G39</f>
-        <v>5.2630875</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="s">
+        <v>8.882775</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B42" s="19" t="n">
+      <c r="B42" s="20" t="n">
         <f aca="false">H39</f>
-        <v>5.2630875</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
+        <v>8.882775</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B43" s="19" t="n">
+      <c r="B43" s="20" t="n">
         <f aca="false">H39*B18</f>
-        <v>2.63154375</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
+        <v>4.4413875</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B44" s="19" t="n">
+      <c r="B44" s="20" t="n">
         <f aca="false">H39*B18*B19</f>
-        <v>0.52630875</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="s">
+        <v>0.8882775</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B45" s="20" t="n">
+      <c r="B45" s="21" t="n">
         <f aca="false">G39</f>
-        <v>1.093125</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="11" t="s">
+        <v>1.8975</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B48" s="15" t="n">
+      <c r="B48" s="16" t="n">
         <f aca="false">B23*12</f>
-        <v>523.5</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B49" s="7" t="n">
+      <c r="B49" s="8" t="n">
         <v>0.04</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B50" s="21" t="n">
+      <c r="B50" s="22" t="n">
         <f aca="false">B48*B49</f>
-        <v>20.94</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
+        <v>40.44</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B51" s="21" t="n">
+      <c r="B51" s="22" t="n">
         <f aca="false">B50*B19</f>
-        <v>4.188</v>
+        <v>8.088</v>
       </c>
     </row>
   </sheetData>
@@ -1436,118 +1440,118 @@
   <dimension ref="A1:A24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="24"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="25" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+    <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="25" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
+    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
+    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="25" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
+    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="s">
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="25" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
+    <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="24" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="s">
+    <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-06-02 20:24:51
</commit_message>
<xml_diff>
--- a/linkedin-inbound-outlook.xlsx
+++ b/linkedin-inbound-outlook.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Model" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Outlook" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Lead &amp; Client Funnel" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="93">
   <si>
     <t xml:space="preserve">Framework OPS — LinkedIn Connection &amp; Inbound Outlook (12 Months)</t>
   </si>
@@ -201,13 +202,112 @@
   </si>
   <si>
     <t xml:space="preserve">Capacity: per Framework OPS plan, realistic delivery ceiling is ~3 Active + 1 Embedded. Pipeline above that is not bookable solo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead → Client Funnel (outreach engine)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base case 75 requests/week (your stated 50-min / 100-lean). Accept rate is blank cold-request, pessimistic &amp; UNMEASURED until 6/3. Green = linked from Model tab; blue = editable here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INPUTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requests / week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accept rate (blank cold)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICP share of accepts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weeks / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow-up → potential lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potential lead → client (close)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery capacity (engagements)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inbound clients / yr (supplemental)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DERIVED (per month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requests / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accepts / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICP accepts / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potential leads / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients / month (steady, pre-ramp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ramp factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potential leads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients signed (mo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative signed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YEAR-1 RESULT @ 75/wk (base case)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients signed, Year 1 (outreach, ramped)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ inbound (supplemental)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL Year-1 clients signed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capped at delivery capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady-state run-rate (clients/yr, yr 2+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO RANGE (annual clients signed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requests/wk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leads/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady clients/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year-1 (ramped)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year-1 capped</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -215,8 +315,9 @@
     <numFmt numFmtId="168" formatCode="0.00%"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,6 +390,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -365,7 +473,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -468,6 +576,78 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -766,7 +946,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -774,7 +954,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -877,7 +1057,7 @@
       </c>
       <c r="B22" s="13" t="n">
         <f aca="false">B7*B9*B8+B11</f>
-        <v>114.333333333333</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -886,7 +1066,7 @@
       </c>
       <c r="B23" s="13" t="n">
         <f aca="false">B7*B9*B8*B10+B11*B12</f>
-        <v>84.25</v>
+        <v>56.625</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -950,19 +1130,19 @@
       </c>
       <c r="B28" s="16" t="n">
         <f aca="false">B27+$B$22</f>
-        <v>670.333333333333</v>
+        <v>633.5</v>
       </c>
       <c r="C28" s="16" t="n">
         <f aca="false">C27+$B$23</f>
-        <v>223.25</v>
+        <v>195.625</v>
       </c>
       <c r="D28" s="17" t="n">
         <f aca="false">C28/B28</f>
-        <v>0.333043262058677</v>
+        <v>0.308800315706393</v>
       </c>
       <c r="E28" s="16" t="n">
         <f aca="false">C28*$B$13</f>
-        <v>122.7875</v>
+        <v>107.59375</v>
       </c>
       <c r="F28" s="18" t="n">
         <f aca="false">IF(A28&lt;=3,$B$14,IF(A28&lt;=6,$B$15,IF(A28&lt;=9,$B$16,$B$17)))</f>
@@ -983,19 +1163,19 @@
       </c>
       <c r="B29" s="16" t="n">
         <f aca="false">B28+$B$22</f>
-        <v>784.666666666667</v>
+        <v>711</v>
       </c>
       <c r="C29" s="16" t="n">
         <f aca="false">C28+$B$23</f>
-        <v>307.5</v>
+        <v>252.25</v>
       </c>
       <c r="D29" s="17" t="n">
         <f aca="false">C29/B29</f>
-        <v>0.391886151231946</v>
+        <v>0.354781997187061</v>
       </c>
       <c r="E29" s="16" t="n">
         <f aca="false">C29*$B$13</f>
-        <v>169.125</v>
+        <v>138.7375</v>
       </c>
       <c r="F29" s="18" t="n">
         <f aca="false">IF(A29&lt;=3,$B$14,IF(A29&lt;=6,$B$15,IF(A29&lt;=9,$B$16,$B$17)))</f>
@@ -1016,19 +1196,19 @@
       </c>
       <c r="B30" s="16" t="n">
         <f aca="false">B29+$B$22</f>
-        <v>899</v>
+        <v>788.5</v>
       </c>
       <c r="C30" s="16" t="n">
         <f aca="false">C29+$B$23</f>
-        <v>391.75</v>
+        <v>308.875</v>
       </c>
       <c r="D30" s="17" t="n">
         <f aca="false">C30/B30</f>
-        <v>0.435761957730812</v>
+        <v>0.391724793912492</v>
       </c>
       <c r="E30" s="16" t="n">
         <f aca="false">C30*$B$13</f>
-        <v>215.4625</v>
+        <v>169.88125</v>
       </c>
       <c r="F30" s="18" t="n">
         <f aca="false">IF(A30&lt;=3,$B$14,IF(A30&lt;=6,$B$15,IF(A30&lt;=9,$B$16,$B$17)))</f>
@@ -1049,19 +1229,19 @@
       </c>
       <c r="B31" s="16" t="n">
         <f aca="false">B30+$B$22</f>
-        <v>1013.33333333333</v>
+        <v>866</v>
       </c>
       <c r="C31" s="16" t="n">
         <f aca="false">C30+$B$23</f>
-        <v>476</v>
+        <v>365.5</v>
       </c>
       <c r="D31" s="17" t="n">
         <f aca="false">C31/B31</f>
-        <v>0.469736842105263</v>
+        <v>0.422055427251732</v>
       </c>
       <c r="E31" s="16" t="n">
         <f aca="false">C31*$B$13</f>
-        <v>261.8</v>
+        <v>201.025</v>
       </c>
       <c r="F31" s="18" t="n">
         <f aca="false">IF(A31&lt;=3,$B$14,IF(A31&lt;=6,$B$15,IF(A31&lt;=9,$B$16,$B$17)))</f>
@@ -1069,11 +1249,11 @@
       </c>
       <c r="G31" s="9" t="n">
         <f aca="false">E31*F31</f>
-        <v>0.2618</v>
+        <v>0.201025</v>
       </c>
       <c r="H31" s="19" t="n">
         <f aca="false">H30+G31</f>
-        <v>0.2618</v>
+        <v>0.201025</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1082,19 +1262,19 @@
       </c>
       <c r="B32" s="16" t="n">
         <f aca="false">B31+$B$22</f>
-        <v>1127.66666666667</v>
+        <v>943.5</v>
       </c>
       <c r="C32" s="16" t="n">
         <f aca="false">C31+$B$23</f>
-        <v>560.25</v>
+        <v>422.125</v>
       </c>
       <c r="D32" s="17" t="n">
         <f aca="false">C32/B32</f>
-        <v>0.496822347029264</v>
+        <v>0.44740328563858</v>
       </c>
       <c r="E32" s="16" t="n">
         <f aca="false">C32*$B$13</f>
-        <v>308.1375</v>
+        <v>232.16875</v>
       </c>
       <c r="F32" s="18" t="n">
         <f aca="false">IF(A32&lt;=3,$B$14,IF(A32&lt;=6,$B$15,IF(A32&lt;=9,$B$16,$B$17)))</f>
@@ -1102,11 +1282,11 @@
       </c>
       <c r="G32" s="9" t="n">
         <f aca="false">E32*F32</f>
-        <v>0.3081375</v>
+        <v>0.23216875</v>
       </c>
       <c r="H32" s="19" t="n">
         <f aca="false">H31+G32</f>
-        <v>0.5699375</v>
+        <v>0.43319375</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1115,19 +1295,19 @@
       </c>
       <c r="B33" s="16" t="n">
         <f aca="false">B32+$B$22</f>
-        <v>1242</v>
+        <v>1021</v>
       </c>
       <c r="C33" s="16" t="n">
         <f aca="false">C32+$B$23</f>
-        <v>644.5</v>
+        <v>478.75</v>
       </c>
       <c r="D33" s="17" t="n">
         <f aca="false">C33/B33</f>
-        <v>0.518921095008052</v>
+        <v>0.468903036238981</v>
       </c>
       <c r="E33" s="16" t="n">
         <f aca="false">C33*$B$13</f>
-        <v>354.475</v>
+        <v>263.3125</v>
       </c>
       <c r="F33" s="18" t="n">
         <f aca="false">IF(A33&lt;=3,$B$14,IF(A33&lt;=6,$B$15,IF(A33&lt;=9,$B$16,$B$17)))</f>
@@ -1135,11 +1315,11 @@
       </c>
       <c r="G33" s="9" t="n">
         <f aca="false">E33*F33</f>
-        <v>0.354475</v>
+        <v>0.2633125</v>
       </c>
       <c r="H33" s="19" t="n">
         <f aca="false">H32+G33</f>
-        <v>0.9244125</v>
+        <v>0.69650625</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1148,19 +1328,19 @@
       </c>
       <c r="B34" s="16" t="n">
         <f aca="false">B33+$B$22</f>
-        <v>1356.33333333333</v>
+        <v>1098.5</v>
       </c>
       <c r="C34" s="16" t="n">
         <f aca="false">C33+$B$23</f>
-        <v>728.75</v>
+        <v>535.375</v>
       </c>
       <c r="D34" s="17" t="n">
         <f aca="false">C34/B34</f>
-        <v>0.537294175473089</v>
+        <v>0.487369139736004</v>
       </c>
       <c r="E34" s="16" t="n">
         <f aca="false">C34*$B$13</f>
-        <v>400.8125</v>
+        <v>294.45625</v>
       </c>
       <c r="F34" s="18" t="n">
         <f aca="false">IF(A34&lt;=3,$B$14,IF(A34&lt;=6,$B$15,IF(A34&lt;=9,$B$16,$B$17)))</f>
@@ -1168,11 +1348,11 @@
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">E34*F34</f>
-        <v>0.801625</v>
+        <v>0.5889125</v>
       </c>
       <c r="H34" s="19" t="n">
         <f aca="false">H33+G34</f>
-        <v>1.7260375</v>
+        <v>1.28541875</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1181,19 +1361,19 @@
       </c>
       <c r="B35" s="16" t="n">
         <f aca="false">B34+$B$22</f>
-        <v>1470.66666666667</v>
+        <v>1176</v>
       </c>
       <c r="C35" s="16" t="n">
         <f aca="false">C34+$B$23</f>
-        <v>813</v>
+        <v>592</v>
       </c>
       <c r="D35" s="17" t="n">
         <f aca="false">C35/B35</f>
-        <v>0.552810516772439</v>
+        <v>0.503401360544218</v>
       </c>
       <c r="E35" s="16" t="n">
         <f aca="false">C35*$B$13</f>
-        <v>447.15</v>
+        <v>325.6</v>
       </c>
       <c r="F35" s="18" t="n">
         <f aca="false">IF(A35&lt;=3,$B$14,IF(A35&lt;=6,$B$15,IF(A35&lt;=9,$B$16,$B$17)))</f>
@@ -1201,11 +1381,11 @@
       </c>
       <c r="G35" s="9" t="n">
         <f aca="false">E35*F35</f>
-        <v>0.8943</v>
+        <v>0.6512</v>
       </c>
       <c r="H35" s="19" t="n">
         <f aca="false">H34+G35</f>
-        <v>2.6203375</v>
+        <v>1.93661875</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1214,19 +1394,19 @@
       </c>
       <c r="B36" s="16" t="n">
         <f aca="false">B35+$B$22</f>
-        <v>1585</v>
+        <v>1253.5</v>
       </c>
       <c r="C36" s="16" t="n">
         <f aca="false">C35+$B$23</f>
-        <v>897.25</v>
+        <v>648.625</v>
       </c>
       <c r="D36" s="17" t="n">
         <f aca="false">C36/B36</f>
-        <v>0.56608832807571</v>
+        <v>0.517451136816913</v>
       </c>
       <c r="E36" s="16" t="n">
         <f aca="false">C36*$B$13</f>
-        <v>493.4875</v>
+        <v>356.74375</v>
       </c>
       <c r="F36" s="18" t="n">
         <f aca="false">IF(A36&lt;=3,$B$14,IF(A36&lt;=6,$B$15,IF(A36&lt;=9,$B$16,$B$17)))</f>
@@ -1234,11 +1414,11 @@
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">E36*F36</f>
-        <v>0.986975</v>
+        <v>0.7134875</v>
       </c>
       <c r="H36" s="19" t="n">
         <f aca="false">H35+G36</f>
-        <v>3.6073125</v>
+        <v>2.65010625</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1247,19 +1427,19 @@
       </c>
       <c r="B37" s="16" t="n">
         <f aca="false">B36+$B$22</f>
-        <v>1699.33333333333</v>
+        <v>1331</v>
       </c>
       <c r="C37" s="16" t="n">
         <f aca="false">C36+$B$23</f>
-        <v>981.5</v>
+        <v>705.25</v>
       </c>
       <c r="D37" s="17" t="n">
         <f aca="false">C37/B37</f>
-        <v>0.577579442918792</v>
+        <v>0.529864763335838</v>
       </c>
       <c r="E37" s="16" t="n">
         <f aca="false">C37*$B$13</f>
-        <v>539.825</v>
+        <v>387.8875</v>
       </c>
       <c r="F37" s="18" t="n">
         <f aca="false">IF(A37&lt;=3,$B$14,IF(A37&lt;=6,$B$15,IF(A37&lt;=9,$B$16,$B$17)))</f>
@@ -1267,11 +1447,11 @@
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">E37*F37</f>
-        <v>1.619475</v>
+        <v>1.1636625</v>
       </c>
       <c r="H37" s="19" t="n">
         <f aca="false">H36+G37</f>
-        <v>5.2267875</v>
+        <v>3.81376875</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1280,19 +1460,19 @@
       </c>
       <c r="B38" s="16" t="n">
         <f aca="false">B37+$B$22</f>
-        <v>1813.66666666667</v>
+        <v>1408.5</v>
       </c>
       <c r="C38" s="16" t="n">
         <f aca="false">C37+$B$23</f>
-        <v>1065.75</v>
+        <v>761.875</v>
       </c>
       <c r="D38" s="17" t="n">
         <f aca="false">C38/B38</f>
-        <v>0.587621760705753</v>
+        <v>0.540912318068868</v>
       </c>
       <c r="E38" s="16" t="n">
         <f aca="false">C38*$B$13</f>
-        <v>586.1625</v>
+        <v>419.03125</v>
       </c>
       <c r="F38" s="18" t="n">
         <f aca="false">IF(A38&lt;=3,$B$14,IF(A38&lt;=6,$B$15,IF(A38&lt;=9,$B$16,$B$17)))</f>
@@ -1300,11 +1480,11 @@
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">E38*F38</f>
-        <v>1.7584875</v>
+        <v>1.25709375</v>
       </c>
       <c r="H38" s="19" t="n">
         <f aca="false">H37+G38</f>
-        <v>6.985275</v>
+        <v>5.0708625</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1313,19 +1493,19 @@
       </c>
       <c r="B39" s="16" t="n">
         <f aca="false">B38+$B$22</f>
-        <v>1928</v>
+        <v>1486</v>
       </c>
       <c r="C39" s="16" t="n">
         <f aca="false">C38+$B$23</f>
-        <v>1150</v>
+        <v>818.5</v>
       </c>
       <c r="D39" s="17" t="n">
         <f aca="false">C39/B39</f>
-        <v>0.596473029045643</v>
+        <v>0.550807537012113</v>
       </c>
       <c r="E39" s="16" t="n">
         <f aca="false">C39*$B$13</f>
-        <v>632.5</v>
+        <v>450.175</v>
       </c>
       <c r="F39" s="18" t="n">
         <f aca="false">IF(A39&lt;=3,$B$14,IF(A39&lt;=6,$B$15,IF(A39&lt;=9,$B$16,$B$17)))</f>
@@ -1333,11 +1513,11 @@
       </c>
       <c r="G39" s="9" t="n">
         <f aca="false">E39*F39</f>
-        <v>1.8975</v>
+        <v>1.350525</v>
       </c>
       <c r="H39" s="19" t="n">
         <f aca="false">H38+G39</f>
-        <v>8.882775</v>
+        <v>6.4213875</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1351,7 +1531,7 @@
       </c>
       <c r="B42" s="20" t="n">
         <f aca="false">H39</f>
-        <v>8.882775</v>
+        <v>6.4213875</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1360,7 +1540,7 @@
       </c>
       <c r="B43" s="20" t="n">
         <f aca="false">H39*B18</f>
-        <v>4.4413875</v>
+        <v>3.21069375</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1369,7 +1549,7 @@
       </c>
       <c r="B44" s="20" t="n">
         <f aca="false">H39*B18*B19</f>
-        <v>0.8882775</v>
+        <v>0.64213875</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1378,7 +1558,7 @@
       </c>
       <c r="B45" s="21" t="n">
         <f aca="false">G39</f>
-        <v>1.8975</v>
+        <v>1.350525</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1392,7 +1572,7 @@
       </c>
       <c r="B48" s="16" t="n">
         <f aca="false">B23*12</f>
-        <v>1011</v>
+        <v>679.5</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1409,7 +1589,7 @@
       </c>
       <c r="B50" s="22" t="n">
         <f aca="false">B48*B49</f>
-        <v>40.44</v>
+        <v>27.18</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1418,7 +1598,7 @@
       </c>
       <c r="B51" s="22" t="n">
         <f aca="false">B50*B19</f>
-        <v>8.088</v>
+        <v>5.436</v>
       </c>
     </row>
   </sheetData>
@@ -1564,4 +1744,560 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E47"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="29"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="31" t="n">
+        <f aca="false">Model!B7</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="32" t="n">
+        <f aca="false">Model!B8</f>
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="32" t="n">
+        <f aca="false">Model!B10</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="33" t="n">
+        <f aca="false">Model!B9</f>
+        <v>4.33333333333333</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="34" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="34" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="38" t="n">
+        <f aca="false">B5*B8</f>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="38" t="n">
+        <f aca="false">B15*B6</f>
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="38" t="n">
+        <f aca="false">B16*B7</f>
+        <v>53.625</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="38" t="n">
+        <f aca="false">B17*B9</f>
+        <v>2.145</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="38" t="n">
+        <f aca="false">B18*B10</f>
+        <v>0.429</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D23" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B23</f>
+        <v>0.0858</v>
+      </c>
+      <c r="E23" s="38" t="n">
+        <f aca="false">0+D23</f>
+        <v>0.0858</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C24" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D24" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B24</f>
+        <v>0.0858</v>
+      </c>
+      <c r="E24" s="38" t="n">
+        <f aca="false">E23+D24</f>
+        <v>0.1716</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C25" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D25" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B25</f>
+        <v>0.1716</v>
+      </c>
+      <c r="E25" s="38" t="n">
+        <f aca="false">E24+D25</f>
+        <v>0.3432</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="40" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C26" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D26" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B26</f>
+        <v>0.1716</v>
+      </c>
+      <c r="E26" s="38" t="n">
+        <f aca="false">E25+D26</f>
+        <v>0.5148</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="40" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C27" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D27" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B27</f>
+        <v>0.2574</v>
+      </c>
+      <c r="E27" s="38" t="n">
+        <f aca="false">E26+D27</f>
+        <v>0.7722</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" s="40" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C28" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D28" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B28</f>
+        <v>0.2574</v>
+      </c>
+      <c r="E28" s="38" t="n">
+        <f aca="false">E27+D28</f>
+        <v>1.0296</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="B29" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C29" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D29" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B29</f>
+        <v>0.3432</v>
+      </c>
+      <c r="E29" s="38" t="n">
+        <f aca="false">E28+D29</f>
+        <v>1.3728</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="B30" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C30" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D30" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B30</f>
+        <v>0.3432</v>
+      </c>
+      <c r="E30" s="38" t="n">
+        <f aca="false">E29+D30</f>
+        <v>1.716</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="B31" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C31" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D31" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B31</f>
+        <v>0.3432</v>
+      </c>
+      <c r="E31" s="38" t="n">
+        <f aca="false">E30+D31</f>
+        <v>2.0592</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="B32" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D32" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B32</f>
+        <v>0.429</v>
+      </c>
+      <c r="E32" s="38" t="n">
+        <f aca="false">E31+D32</f>
+        <v>2.4882</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="B33" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D33" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B33</f>
+        <v>0.429</v>
+      </c>
+      <c r="E33" s="38" t="n">
+        <f aca="false">E32+D33</f>
+        <v>2.9172</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B34" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="38" t="n">
+        <f aca="false">$B$18</f>
+        <v>2.145</v>
+      </c>
+      <c r="D34" s="38" t="n">
+        <f aca="false">$B$18*$B$10*B34</f>
+        <v>0.429</v>
+      </c>
+      <c r="E34" s="38" t="n">
+        <f aca="false">E33+D34</f>
+        <v>3.3462</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="37" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="B37" s="41" t="n">
+        <f aca="false">E34</f>
+        <v>3.3462</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" s="41" t="n">
+        <f aca="false">B12</f>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="B39" s="41" t="n">
+        <f aca="false">E34+B12</f>
+        <v>4.0462</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="41" t="n">
+        <f aca="false">MIN(E34+B12,B11)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="B41" s="41" t="n">
+        <f aca="false">B18*B10*12+B12</f>
+        <v>5.848</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="37" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="42" t="n">
+        <v>50</v>
+      </c>
+      <c r="B45" s="43" t="n">
+        <f aca="false">50*$B$6*$B$7*$B$9*$B$8*12</f>
+        <v>17.16</v>
+      </c>
+      <c r="C45" s="43" t="n">
+        <f aca="false">B45*$B$10+$B$12</f>
+        <v>4.132</v>
+      </c>
+      <c r="D45" s="43" t="n">
+        <f aca="false">C45*0.65</f>
+        <v>2.6858</v>
+      </c>
+      <c r="E45" s="41" t="n">
+        <f aca="false">MIN(D45,$B$11)</f>
+        <v>2.6858</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="42" t="n">
+        <v>75</v>
+      </c>
+      <c r="B46" s="43" t="n">
+        <f aca="false">75*$B$6*$B$7*$B$9*$B$8*12</f>
+        <v>25.74</v>
+      </c>
+      <c r="C46" s="43" t="n">
+        <f aca="false">B46*$B$10+$B$12</f>
+        <v>5.848</v>
+      </c>
+      <c r="D46" s="43" t="n">
+        <f aca="false">C46*0.65</f>
+        <v>3.8012</v>
+      </c>
+      <c r="E46" s="41" t="n">
+        <f aca="false">MIN(D46,$B$11)</f>
+        <v>3.8012</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="B47" s="43" t="n">
+        <f aca="false">100*$B$6*$B$7*$B$9*$B$8*12</f>
+        <v>34.32</v>
+      </c>
+      <c r="C47" s="43" t="n">
+        <f aca="false">B47*$B$10+$B$12</f>
+        <v>7.564</v>
+      </c>
+      <c r="D47" s="43" t="n">
+        <f aca="false">C47*0.65</f>
+        <v>4.9166</v>
+      </c>
+      <c r="E47" s="41" t="n">
+        <f aca="false">MIN(D47,$B$11)</f>
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>